<commit_message>
Added to it now
</commit_message>
<xml_diff>
--- a/Data/EX/students.xlsx
+++ b/Data/EX/students.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Repositories\kjsitfeedback\Data\EX\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D45CD29-CF75-463A-A386-2F349F812CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ADC946D-075F-49C4-881B-66AD5BC7C170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3125" uniqueCount="1807">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3125" uniqueCount="1809">
   <si>
     <t>First Name</t>
   </si>
@@ -5453,13 +5453,19 @@
   </si>
   <si>
     <t>7EXTCB_42</t>
+  </si>
+  <si>
+    <t>abhijit.gurav@somaiya.edu</t>
+  </si>
+  <si>
+    <t>abhijit.gurav</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5504,6 +5510,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF212529"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -5553,12 +5567,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5617,8 +5632,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal 4" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
@@ -12118,11 +12137,11 @@
       <c r="B214" s="5" t="s">
         <v>643</v>
       </c>
-      <c r="C214" s="9" t="s">
-        <v>389</v>
+      <c r="C214" s="22" t="s">
+        <v>1807</v>
       </c>
       <c r="D214" s="9" t="s">
-        <v>1201</v>
+        <v>1808</v>
       </c>
       <c r="E214" s="8" t="s">
         <v>1643</v>
@@ -16880,6 +16899,9 @@
     <row r="388" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="389" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C214" r:id="rId1" xr:uid="{31097FA1-DF6C-4324-B576-6D4937BD95E1}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>